<commit_message>
JOBS: schedule weekly pick-forensics Slack digest (Sun 17:30 PT)
com.swingtrade.forensics-weekly runs pick_forensics.py --slack --days 14 every Sunday
17:30 PT (after weekly-diagnostics 17:00 + week's trades closed/labeled). Posts the 14d
verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack automatically.
Loaded in launchd; lint OK.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-05-31.xlsx
+++ b/cache/open_items_2026-05-31.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N240"/>
+  <dimension ref="A1:N241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -12020,13 +12020,13 @@
       </c>
       <c r="N202" s="8" t="inlineStr"/>
     </row>
-    <row r="203" ht="75" customHeight="1">
+    <row r="203" ht="45" customHeight="1">
       <c r="A203" s="2" t="n">
         <v>202</v>
       </c>
       <c r="B203" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
+          <t>FORENSICS-WEEKLY-SLACK</t>
         </is>
       </c>
       <c r="C203" s="10" t="inlineStr">
@@ -12036,39 +12036,27 @@
       </c>
       <c r="D203" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Notifications / Audit</t>
         </is>
       </c>
       <c r="E203" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Weekly pick-forensics Slack digest</t>
         </is>
       </c>
       <c r="F203" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
         </is>
       </c>
       <c r="G203" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
-        </is>
-      </c>
-      <c r="H203" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I203" s="5" t="inlineStr">
-        <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
-        </is>
-      </c>
-      <c r="J203" s="5" t="inlineStr">
-        <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
-        </is>
-      </c>
+          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr"/>
+      <c r="I203" s="5" t="inlineStr"/>
+      <c r="J203" s="5" t="inlineStr"/>
       <c r="K203" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -12076,27 +12064,23 @@
       </c>
       <c r="L203" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M203" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N203" s="8" t="inlineStr">
-        <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="204" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N203" s="8" t="inlineStr"/>
+    </row>
+    <row r="204" ht="75" customHeight="1">
       <c r="A204" s="2" t="n">
         <v>203</v>
       </c>
       <c r="B204" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C204" s="10" t="inlineStr">
@@ -12106,37 +12090,37 @@
       </c>
       <c r="D204" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E204" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F204" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G204" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I204" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J204" s="5" t="inlineStr">
         <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K204" s="12" t="inlineStr">
@@ -12146,17 +12130,17 @@
       </c>
       <c r="L204" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M204" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N204" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
         </is>
       </c>
     </row>
@@ -12166,7 +12150,7 @@
       </c>
       <c r="B205" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C205" s="10" t="inlineStr">
@@ -12181,32 +12165,32 @@
       </c>
       <c r="E205" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F205" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G205" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I205" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J205" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K205" s="12" t="inlineStr">
@@ -12226,7 +12210,7 @@
       </c>
       <c r="N205" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -12236,7 +12220,7 @@
       </c>
       <c r="B206" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C206" s="10" t="inlineStr">
@@ -12251,32 +12235,32 @@
       </c>
       <c r="E206" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F206" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G206" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I206" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J206" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K206" s="12" t="inlineStr">
@@ -12296,7 +12280,7 @@
       </c>
       <c r="N206" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
         </is>
       </c>
     </row>
@@ -12306,7 +12290,7 @@
       </c>
       <c r="B207" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>OPS-4</t>
         </is>
       </c>
       <c r="C207" s="10" t="inlineStr">
@@ -12321,32 +12305,32 @@
       </c>
       <c r="E207" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F207" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G207" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I207" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J207" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K207" s="12" t="inlineStr">
@@ -12356,27 +12340,27 @@
       </c>
       <c r="L207" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M207" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N207" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="208" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="60" customHeight="1">
       <c r="A208" s="2" t="n">
         <v>207</v>
       </c>
       <c r="B208" s="3" t="inlineStr">
         <is>
-          <t>SCAN-FAILURE-ALERT</t>
+          <t>OPS-5</t>
         </is>
       </c>
       <c r="C208" s="10" t="inlineStr">
@@ -12386,27 +12370,39 @@
       </c>
       <c r="D208" s="5" t="inlineStr">
         <is>
-          <t>Ops / Alerts</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E208" s="6" t="inlineStr">
         <is>
-          <t>Scan-failure + EODHD-quota Slack alert</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F208" s="5" t="inlineStr">
         <is>
-          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G208" s="5" t="inlineStr">
         <is>
-          <t>swing_trade.py exit hook</t>
-        </is>
-      </c>
-      <c r="H208" s="2" t="inlineStr"/>
-      <c r="I208" s="5" t="inlineStr"/>
-      <c r="J208" s="5" t="inlineStr"/>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I208" s="5" t="inlineStr">
+        <is>
+          <t>Win: fast iteration on report templates.</t>
+        </is>
+      </c>
+      <c r="J208" s="5" t="inlineStr">
+        <is>
+          <t>Trivial CLI wrapper.</t>
+        </is>
+      </c>
       <c r="K208" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -12414,15 +12410,19 @@
       </c>
       <c r="L208" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M208" s="3" t="inlineStr">
         <is>
-          <t>0dc7675ee</t>
-        </is>
-      </c>
-      <c r="N208" s="8" t="inlineStr"/>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N208" s="8" t="inlineStr">
+        <is>
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="209" ht="45" customHeight="1">
       <c r="A209" s="2" t="n">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="B209" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
+          <t>SCAN-FAILURE-ALERT</t>
         </is>
       </c>
       <c r="C209" s="10" t="inlineStr">
@@ -12440,22 +12440,22 @@
       </c>
       <c r="D209" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Alerts</t>
         </is>
       </c>
       <c r="E209" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot: load or retire</t>
+          <t>Scan-failure + EODHD-quota Slack alert</t>
         </is>
       </c>
       <c r="F209" s="5" t="inlineStr">
         <is>
-          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
+          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
         </is>
       </c>
       <c r="G209" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd</t>
+          <t>swing_trade.py exit hook</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr"/>
@@ -12478,13 +12478,13 @@
       </c>
       <c r="N209" s="8" t="inlineStr"/>
     </row>
-    <row r="210" ht="150" customHeight="1">
+    <row r="210" ht="45" customHeight="1">
       <c r="A210" s="2" t="n">
         <v>209</v>
       </c>
       <c r="B210" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
         </is>
       </c>
       <c r="C210" s="10" t="inlineStr">
@@ -12494,31 +12494,27 @@
       </c>
       <c r="D210" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E210" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Decide momentum-snapshot: load or retire</t>
         </is>
       </c>
       <c r="F210" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
         </is>
       </c>
       <c r="G210" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+          <t>infra/launchd</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr"/>
       <c r="I210" s="5" t="inlineStr"/>
-      <c r="J210" s="5" t="inlineStr">
-        <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
-        </is>
-      </c>
+      <c r="J210" s="5" t="inlineStr"/>
       <c r="K210" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -12526,27 +12522,23 @@
       </c>
       <c r="L210" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M210" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
-        </is>
-      </c>
-      <c r="N210" s="8" t="inlineStr">
-        <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="211" ht="45" customHeight="1">
+          <t>0dc7675ee</t>
+        </is>
+      </c>
+      <c r="N210" s="8" t="inlineStr"/>
+    </row>
+    <row r="211" ht="150" customHeight="1">
       <c r="A211" s="2" t="n">
         <v>210</v>
       </c>
       <c r="B211" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-1</t>
+          <t>PERF-7b</t>
         </is>
       </c>
       <c r="C211" s="10" t="inlineStr">
@@ -12556,27 +12548,31 @@
       </c>
       <c r="D211" s="5" t="inlineStr">
         <is>
-          <t>Sharpe Roadmap</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E211" s="6" t="inlineStr">
         <is>
-          <t>Sharpe gate in momentum detector</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F211" s="5" t="inlineStr">
         <is>
-          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G211" s="5" t="inlineStr">
         <is>
-          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr"/>
       <c r="I211" s="5" t="inlineStr"/>
-      <c r="J211" s="5" t="inlineStr"/>
+      <c r="J211" s="5" t="inlineStr">
+        <is>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+        </is>
+      </c>
       <c r="K211" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -12584,15 +12580,19 @@
       </c>
       <c r="L211" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M211" s="3" t="inlineStr">
         <is>
-          <t>dbbd6b5f6</t>
-        </is>
-      </c>
-      <c r="N211" s="8" t="inlineStr"/>
+          <t>cf30df858</t>
+        </is>
+      </c>
+      <c r="N211" s="8" t="inlineStr">
+        <is>
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="45" customHeight="1">
       <c r="A212" s="2" t="n">
@@ -12600,7 +12600,7 @@
       </c>
       <c r="B212" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-10</t>
+          <t>SHARPE-1</t>
         </is>
       </c>
       <c r="C212" s="10" t="inlineStr">
@@ -12615,17 +12615,17 @@
       </c>
       <c r="E212" s="6" t="inlineStr">
         <is>
-          <t>Sharpe alerts for watchlist</t>
+          <t>Sharpe gate in momentum detector</t>
         </is>
       </c>
       <c r="F212" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
         </is>
       </c>
       <c r="G212" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
+          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr"/>
@@ -12654,7 +12654,7 @@
       </c>
       <c r="B213" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-11</t>
+          <t>SHARPE-10</t>
         </is>
       </c>
       <c r="C213" s="10" t="inlineStr">
@@ -12669,17 +12669,17 @@
       </c>
       <c r="E213" s="6" t="inlineStr">
         <is>
-          <t>Per-trade Sharpe attribution</t>
+          <t>Sharpe alerts for watchlist</t>
         </is>
       </c>
       <c r="F213" s="5" t="inlineStr">
         <is>
-          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G213" s="5" t="inlineStr">
         <is>
-          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
+          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr"/>
@@ -12708,7 +12708,7 @@
       </c>
       <c r="B214" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-12</t>
+          <t>SHARPE-11</t>
         </is>
       </c>
       <c r="C214" s="10" t="inlineStr">
@@ -12723,17 +12723,17 @@
       </c>
       <c r="E214" s="6" t="inlineStr">
         <is>
-          <t>Sharpe consistency check</t>
+          <t>Per-trade Sharpe attribution</t>
         </is>
       </c>
       <c r="F214" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
         </is>
       </c>
       <c r="G214" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
+          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr"/>
@@ -12762,7 +12762,7 @@
       </c>
       <c r="B215" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-2</t>
+          <t>SHARPE-12</t>
         </is>
       </c>
       <c r="C215" s="10" t="inlineStr">
@@ -12777,17 +12777,17 @@
       </c>
       <c r="E215" s="6" t="inlineStr">
         <is>
-          <t>Sharpe column in v2 dashboard</t>
+          <t>Sharpe consistency check</t>
         </is>
       </c>
       <c r="F215" s="5" t="inlineStr">
         <is>
-          <t>Surface 126d Sharpe per ticker as sortable column</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G215" s="5" t="inlineStr">
         <is>
-          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
+          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr"/>
@@ -12816,7 +12816,7 @@
       </c>
       <c r="B216" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-3</t>
+          <t>SHARPE-2</t>
         </is>
       </c>
       <c r="C216" s="10" t="inlineStr">
@@ -12831,17 +12831,17 @@
       </c>
       <c r="E216" s="6" t="inlineStr">
         <is>
-          <t>Per-stock Sharpe by regime</t>
+          <t>Sharpe column in v2 dashboard</t>
         </is>
       </c>
       <c r="F216" s="5" t="inlineStr">
         <is>
-          <t>Decompose per-stock Sharpe by historical regime tags</t>
+          <t>Surface 126d Sharpe per ticker as sortable column</t>
         </is>
       </c>
       <c r="G216" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
+          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr"/>
@@ -12870,7 +12870,7 @@
       </c>
       <c r="B217" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-4</t>
+          <t>SHARPE-3</t>
         </is>
       </c>
       <c r="C217" s="10" t="inlineStr">
@@ -12885,17 +12885,17 @@
       </c>
       <c r="E217" s="6" t="inlineStr">
         <is>
-          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
+          <t>Per-stock Sharpe by regime</t>
         </is>
       </c>
       <c r="F217" s="5" t="inlineStr">
         <is>
-          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
+          <t>Decompose per-stock Sharpe by historical regime tags</t>
         </is>
       </c>
       <c r="G217" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
+          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr"/>
@@ -12924,7 +12924,7 @@
       </c>
       <c r="B218" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-5</t>
+          <t>SHARPE-4</t>
         </is>
       </c>
       <c r="C218" s="10" t="inlineStr">
@@ -12939,17 +12939,17 @@
       </c>
       <c r="E218" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-weighted position sizing</t>
+          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
         </is>
       </c>
       <c r="F218" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
         </is>
       </c>
       <c r="G218" s="5" t="inlineStr">
         <is>
-          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr"/>
@@ -12978,7 +12978,7 @@
       </c>
       <c r="B219" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-6</t>
+          <t>SHARPE-5</t>
         </is>
       </c>
       <c r="C219" s="10" t="inlineStr">
@@ -12993,17 +12993,17 @@
       </c>
       <c r="E219" s="6" t="inlineStr">
         <is>
-          <t>Portfolio Sharpe KPI vs target</t>
+          <t>Sharpe-weighted position sizing</t>
         </is>
       </c>
       <c r="F219" s="5" t="inlineStr">
         <is>
-          <t>Annualized Sharpe target tracking + gap report</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G219" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
+          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr"/>
@@ -13032,7 +13032,7 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-7</t>
+          <t>SHARPE-6</t>
         </is>
       </c>
       <c r="C220" s="10" t="inlineStr">
@@ -13047,17 +13047,17 @@
       </c>
       <c r="E220" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-based stop sizing</t>
+          <t>Portfolio Sharpe KPI vs target</t>
         </is>
       </c>
       <c r="F220" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Annualized Sharpe target tracking + gap report</t>
         </is>
       </c>
       <c r="G220" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr"/>
@@ -13086,7 +13086,7 @@
       </c>
       <c r="B221" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-8</t>
+          <t>SHARPE-7</t>
         </is>
       </c>
       <c r="C221" s="10" t="inlineStr">
@@ -13101,17 +13101,17 @@
       </c>
       <c r="E221" s="6" t="inlineStr">
         <is>
-          <t>Sortino computation alongside Sharpe</t>
+          <t>Sharpe-based stop sizing</t>
         </is>
       </c>
       <c r="F221" s="5" t="inlineStr">
         <is>
-          <t>Downside-only vol denominator added everywhere</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G221" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
+          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr"/>
@@ -13140,7 +13140,7 @@
       </c>
       <c r="B222" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-9</t>
+          <t>SHARPE-8</t>
         </is>
       </c>
       <c r="C222" s="10" t="inlineStr">
@@ -13155,17 +13155,17 @@
       </c>
       <c r="E222" s="6" t="inlineStr">
         <is>
-          <t>SPY-Sharpe regime cross-validation</t>
+          <t>Sortino computation alongside Sharpe</t>
         </is>
       </c>
       <c r="F222" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Downside-only vol denominator added everywhere</t>
         </is>
       </c>
       <c r="G222" s="5" t="inlineStr">
         <is>
-          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
+          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr"/>
@@ -13188,13 +13188,13 @@
       </c>
       <c r="N222" s="8" t="inlineStr"/>
     </row>
-    <row r="223" ht="120" customHeight="1">
+    <row r="223" ht="45" customHeight="1">
       <c r="A223" s="2" t="n">
         <v>222</v>
       </c>
       <c r="B223" s="3" t="inlineStr">
         <is>
-          <t>CONVICTION-TIER-WIRE</t>
+          <t>SHARPE-9</t>
         </is>
       </c>
       <c r="C223" s="10" t="inlineStr">
@@ -13204,39 +13204,27 @@
       </c>
       <c r="D223" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Conviction</t>
+          <t>Sharpe Roadmap</t>
         </is>
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>Conviction tier: simplified to score-band only</t>
+          <t>SPY-Sharpe regime cross-validation</t>
         </is>
       </c>
       <c r="F223" s="5" t="inlineStr">
         <is>
-          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G223" s="5" t="inlineStr">
         <is>
-          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
-        </is>
-      </c>
-      <c r="H223" s="2" t="inlineStr">
-        <is>
-          <t>2-4 hrs + backtest validation</t>
-        </is>
-      </c>
-      <c r="I223" s="5" t="inlineStr">
-        <is>
-          <t>Medium — changes live size or eliminates a layer</t>
-        </is>
-      </c>
-      <c r="J223" s="5" t="inlineStr">
-        <is>
-          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
-        </is>
-      </c>
+          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr"/>
+      <c r="I223" s="5" t="inlineStr"/>
+      <c r="J223" s="5" t="inlineStr"/>
       <c r="K223" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13244,27 +13232,23 @@
       </c>
       <c r="L223" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M223" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N223" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
-        </is>
-      </c>
-    </row>
-    <row r="224" ht="75" customHeight="1">
+          <t>dbbd6b5f6</t>
+        </is>
+      </c>
+      <c r="N223" s="8" t="inlineStr"/>
+    </row>
+    <row r="224" ht="120" customHeight="1">
       <c r="A224" s="2" t="n">
         <v>223</v>
       </c>
       <c r="B224" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-Q-AB</t>
+          <t>CONVICTION-TIER-WIRE</t>
         </is>
       </c>
       <c r="C224" s="10" t="inlineStr">
@@ -13274,27 +13258,39 @@
       </c>
       <c r="D224" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Gates</t>
+          <t>Strategy / Conviction</t>
         </is>
       </c>
       <c r="E224" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional entry_quality A/B</t>
+          <t>Conviction tier: simplified to score-band only</t>
         </is>
       </c>
       <c r="F224" s="5" t="inlineStr">
         <is>
-          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
+          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
         </is>
       </c>
       <c r="G224" s="5" t="inlineStr">
         <is>
-          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
-        </is>
-      </c>
-      <c r="H224" s="2" t="inlineStr"/>
-      <c r="I224" s="5" t="inlineStr"/>
-      <c r="J224" s="5" t="inlineStr"/>
+          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>2-4 hrs + backtest validation</t>
+        </is>
+      </c>
+      <c r="I224" s="5" t="inlineStr">
+        <is>
+          <t>Medium — changes live size or eliminates a layer</t>
+        </is>
+      </c>
+      <c r="J224" s="5" t="inlineStr">
+        <is>
+          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
+        </is>
+      </c>
       <c r="K224" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13302,23 +13298,27 @@
       </c>
       <c r="L224" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M224" s="3" t="inlineStr">
         <is>
-          <t>07c3af6a3</t>
-        </is>
-      </c>
-      <c r="N224" s="8" t="inlineStr"/>
-    </row>
-    <row r="225" ht="120" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N224" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="75" customHeight="1">
       <c r="A225" s="2" t="n">
         <v>224</v>
       </c>
       <c r="B225" s="3" t="inlineStr">
         <is>
-          <t>UI-STRAT-1</t>
+          <t>ENTRY-Q-AB</t>
         </is>
       </c>
       <c r="C225" s="10" t="inlineStr">
@@ -13328,22 +13328,22 @@
       </c>
       <c r="D225" s="5" t="inlineStr">
         <is>
-          <t>Strategy Lab</t>
+          <t>Strategy / Gates</t>
         </is>
       </c>
       <c r="E225" s="6" t="inlineStr">
         <is>
-          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
+          <t>Regime-conditional entry_quality A/B</t>
         </is>
       </c>
       <c r="F225" s="5" t="inlineStr">
         <is>
-          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
+          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
         </is>
       </c>
       <c r="G225" s="5" t="inlineStr">
         <is>
-          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
+          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
         </is>
       </c>
       <c r="H225" s="2" t="inlineStr"/>
@@ -13356,23 +13356,23 @@
       </c>
       <c r="L225" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M225" s="3" t="inlineStr">
         <is>
-          <t>93ec11842</t>
+          <t>07c3af6a3</t>
         </is>
       </c>
       <c r="N225" s="8" t="inlineStr"/>
     </row>
-    <row r="226" ht="105" customHeight="1">
+    <row r="226" ht="120" customHeight="1">
       <c r="A226" s="2" t="n">
         <v>225</v>
       </c>
       <c r="B226" s="3" t="inlineStr">
         <is>
-          <t>TRACKER-BUY-FILTER</t>
+          <t>UI-STRAT-1</t>
         </is>
       </c>
       <c r="C226" s="10" t="inlineStr">
@@ -13382,31 +13382,27 @@
       </c>
       <c r="D226" s="5" t="inlineStr">
         <is>
-          <t>Tracker/Feedback Loop</t>
+          <t>Strategy Lab</t>
         </is>
       </c>
       <c r="E226" s="6" t="inlineStr">
         <is>
-          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
+          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
         </is>
       </c>
       <c r="F226" s="5" t="inlineStr">
         <is>
-          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
+          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
         </is>
       </c>
       <c r="G226" s="5" t="inlineStr">
         <is>
-          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr"/>
       <c r="I226" s="5" t="inlineStr"/>
-      <c r="J226" s="5" t="inlineStr">
-        <is>
-          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
-        </is>
-      </c>
+      <c r="J226" s="5" t="inlineStr"/>
       <c r="K226" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13414,27 +13410,23 @@
       </c>
       <c r="L226" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M226" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N226" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="227" ht="135" customHeight="1">
+          <t>93ec11842</t>
+        </is>
+      </c>
+      <c r="N226" s="8" t="inlineStr"/>
+    </row>
+    <row r="227" ht="105" customHeight="1">
       <c r="A227" s="2" t="n">
         <v>226</v>
       </c>
       <c r="B227" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
+          <t>TRACKER-BUY-FILTER</t>
         </is>
       </c>
       <c r="C227" s="10" t="inlineStr">
@@ -13444,37 +13436,29 @@
       </c>
       <c r="D227" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Tracker/Feedback Loop</t>
         </is>
       </c>
       <c r="E227" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
         </is>
       </c>
       <c r="F227" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
         </is>
       </c>
       <c r="G227" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
-        </is>
-      </c>
-      <c r="H227" s="2" t="inlineStr">
-        <is>
-          <t>1-2 hrs</t>
-        </is>
-      </c>
-      <c r="I227" s="5" t="inlineStr">
-        <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
-        </is>
-      </c>
+          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr"/>
+      <c r="I227" s="5" t="inlineStr"/>
       <c r="J227" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
         </is>
       </c>
       <c r="K227" s="12" t="inlineStr">
@@ -13484,27 +13468,27 @@
       </c>
       <c r="L227" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M227" s="3" t="inlineStr">
         <is>
-          <t>42c36ef91</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N227" s="8" t="inlineStr">
         <is>
-          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="228" ht="45" customHeight="1">
+          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="135" customHeight="1">
       <c r="A228" s="2" t="n">
         <v>227</v>
       </c>
       <c r="B228" s="3" t="inlineStr">
         <is>
-          <t>STOCKSMITH-BOOK-RISK</t>
+          <t>MOD-1</t>
         </is>
       </c>
       <c r="C228" s="10" t="inlineStr">
@@ -13514,27 +13498,39 @@
       </c>
       <c r="D228" s="5" t="inlineStr">
         <is>
-          <t>V2 Dashboard / Risk</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E228" s="6" t="inlineStr">
         <is>
-          <t>Book Risk surface + per-lens analytics (§6)</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F228" s="5" t="inlineStr">
         <is>
-          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G228" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
-        </is>
-      </c>
-      <c r="H228" s="2" t="inlineStr"/>
-      <c r="I228" s="5" t="inlineStr"/>
-      <c r="J228" s="5" t="inlineStr"/>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I228" s="5" t="inlineStr">
+        <is>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
+        </is>
+      </c>
+      <c r="J228" s="5" t="inlineStr">
+        <is>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+        </is>
+      </c>
       <c r="K228" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13542,23 +13538,27 @@
       </c>
       <c r="L228" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M228" s="3" t="inlineStr">
         <is>
-          <t>50cace567</t>
-        </is>
-      </c>
-      <c r="N228" s="8" t="inlineStr"/>
-    </row>
-    <row r="229" ht="120" customHeight="1">
+          <t>42c36ef91</t>
+        </is>
+      </c>
+      <c r="N228" s="8" t="inlineStr">
+        <is>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="45" customHeight="1">
       <c r="A229" s="2" t="n">
         <v>228</v>
       </c>
       <c r="B229" s="3" t="inlineStr">
         <is>
-          <t>RECENCY-FLOOR</t>
+          <t>STOCKSMITH-BOOK-RISK</t>
         </is>
       </c>
       <c r="C229" s="10" t="inlineStr">
@@ -13568,31 +13568,27 @@
       </c>
       <c r="D229" s="5" t="inlineStr">
         <is>
-          <t>Validation Hygiene</t>
+          <t>V2 Dashboard / Risk</t>
         </is>
       </c>
       <c r="E229" s="6" t="inlineStr">
         <is>
-          <t>_validations needs recency floor — auto-revert stale boosts</t>
+          <t>Book Risk surface + per-lens analytics (§6)</t>
         </is>
       </c>
       <c r="F229" s="5" t="inlineStr">
         <is>
-          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
+          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
         </is>
       </c>
       <c r="G229" s="5" t="inlineStr">
         <is>
-          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
+          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr"/>
       <c r="I229" s="5" t="inlineStr"/>
-      <c r="J229" s="5" t="inlineStr">
-        <is>
-          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
-        </is>
-      </c>
+      <c r="J229" s="5" t="inlineStr"/>
       <c r="K229" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13600,27 +13596,23 @@
       </c>
       <c r="L229" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="M229" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N229" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="230" ht="60" customHeight="1">
+          <t>50cace567</t>
+        </is>
+      </c>
+      <c r="N229" s="8" t="inlineStr"/>
+    </row>
+    <row r="230" ht="120" customHeight="1">
       <c r="A230" s="2" t="n">
         <v>229</v>
       </c>
       <c r="B230" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-TAB</t>
+          <t>RECENCY-FLOOR</t>
         </is>
       </c>
       <c r="C230" s="10" t="inlineStr">
@@ -13630,27 +13622,31 @@
       </c>
       <c r="D230" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Momentum</t>
+          <t>Validation Hygiene</t>
         </is>
       </c>
       <c r="E230" s="6" t="inlineStr">
         <is>
-          <t>New 🚀 Momentum workspace tab</t>
+          <t>_validations needs recency floor — auto-revert stale boosts</t>
         </is>
       </c>
       <c r="F230" s="5" t="inlineStr">
         <is>
-          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
+          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
         </is>
       </c>
       <c r="G230" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
+          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr"/>
       <c r="I230" s="5" t="inlineStr"/>
-      <c r="J230" s="5" t="inlineStr"/>
+      <c r="J230" s="5" t="inlineStr">
+        <is>
+          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
+        </is>
+      </c>
       <c r="K230" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13658,15 +13654,19 @@
       </c>
       <c r="L230" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M230" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N230" s="8" t="inlineStr"/>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N230" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="60" customHeight="1">
       <c r="A231" s="2" t="n">
@@ -13674,7 +13674,7 @@
       </c>
       <c r="B231" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-QUICK-PANELS</t>
+          <t>MOMENTUM-TAB</t>
         </is>
       </c>
       <c r="C231" s="10" t="inlineStr">
@@ -13684,22 +13684,22 @@
       </c>
       <c r="D231" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Signal Scanner</t>
+          <t>Workspaces / Momentum</t>
         </is>
       </c>
       <c r="E231" s="6" t="inlineStr">
         <is>
-          <t>5 quick-glance panels above watchlist table</t>
+          <t>New 🚀 Momentum workspace tab</t>
         </is>
       </c>
       <c r="F231" s="5" t="inlineStr">
         <is>
-          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
+          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
         </is>
       </c>
       <c r="G231" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr"/>
@@ -13717,60 +13717,48 @@
       </c>
       <c r="M231" s="3" t="inlineStr">
         <is>
-          <t>dfbe955fe</t>
+          <t>27fd646b1</t>
         </is>
       </c>
       <c r="N231" s="8" t="inlineStr"/>
     </row>
-    <row r="232" ht="45" customHeight="1">
+    <row r="232" ht="60" customHeight="1">
       <c r="A232" s="2" t="n">
         <v>231</v>
       </c>
       <c r="B232" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C232" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>SCANNER-QUICK-PANELS</t>
+        </is>
+      </c>
+      <c r="C232" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D232" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Workspaces / Signal Scanner</t>
         </is>
       </c>
       <c r="E232" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>5 quick-glance panels above watchlist table</t>
         </is>
       </c>
       <c r="F232" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
         </is>
       </c>
       <c r="G232" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
-        </is>
-      </c>
-      <c r="H232" s="2" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="I232" s="5" t="inlineStr">
-        <is>
-          <t>Win: persistence works; no silent overwrites.</t>
-        </is>
-      </c>
-      <c r="J232" s="5" t="inlineStr">
-        <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
-        </is>
-      </c>
+          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr"/>
+      <c r="I232" s="5" t="inlineStr"/>
+      <c r="J232" s="5" t="inlineStr"/>
       <c r="K232" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13778,15 +13766,15 @@
       </c>
       <c r="L232" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M232" s="3" t="inlineStr"/>
-      <c r="N232" s="8" t="inlineStr">
-        <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="M232" s="3" t="inlineStr">
+        <is>
+          <t>dfbe955fe</t>
+        </is>
+      </c>
+      <c r="N232" s="8" t="inlineStr"/>
     </row>
     <row r="233" ht="45" customHeight="1">
       <c r="A233" s="2" t="n">
@@ -13794,7 +13782,7 @@
       </c>
       <c r="B233" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="C233" s="13" t="inlineStr">
@@ -13809,32 +13797,32 @@
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F233" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G233" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H233" s="2" t="inlineStr">
         <is>
-          <t>verified (no change needed)</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I233" s="5" t="inlineStr">
         <is>
-          <t>Win: confirms infrastructure still healthy.</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J233" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
         </is>
       </c>
       <c r="K233" s="12" t="inlineStr">
@@ -13850,7 +13838,7 @@
       <c r="M233" s="3" t="inlineStr"/>
       <c r="N233" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
         </is>
       </c>
     </row>
@@ -13860,7 +13848,7 @@
       </c>
       <c r="B234" s="3" t="inlineStr">
         <is>
-          <t>UI-3</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C234" s="13" t="inlineStr">
@@ -13870,35 +13858,39 @@
       </c>
       <c r="D234" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E234" s="6" t="inlineStr">
         <is>
-          <t>Remove emoji icons from Thesis + Research labels</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F234" s="5" t="inlineStr">
         <is>
-          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G234" s="5" t="inlineStr">
         <is>
-          <t>Removed emojis from FD sub-tab nav + section headers.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I234" s="5" t="inlineStr">
         <is>
-          <t>Low / cosmetic</t>
-        </is>
-      </c>
-      <c r="J234" s="5" t="inlineStr"/>
+          <t>Win: confirms infrastructure still healthy.</t>
+        </is>
+      </c>
+      <c r="J234" s="5" t="inlineStr">
+        <is>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
       <c r="K234" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -13906,17 +13898,13 @@
       </c>
       <c r="L234" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="M234" s="3" t="inlineStr">
-        <is>
-          <t>24fd7c273</t>
-        </is>
-      </c>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M234" s="3" t="inlineStr"/>
       <c r="N234" s="8" t="inlineStr">
         <is>
-          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
         </is>
       </c>
     </row>
@@ -13926,59 +13914,63 @@
       </c>
       <c r="B235" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
-        </is>
-      </c>
-      <c r="C235" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>UI-3</t>
+        </is>
+      </c>
+      <c r="C235" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D235" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E235" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Remove emoji icons from Thesis + Research labels</t>
         </is>
       </c>
       <c r="F235" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
         </is>
       </c>
       <c r="G235" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+          <t>Removed emojis from FD sub-tab nav + section headers.</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr">
         <is>
-          <t>5 min after answer</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I235" s="5" t="inlineStr">
         <is>
-          <t>Win: -671 lines.</t>
-        </is>
-      </c>
-      <c r="J235" s="5" t="inlineStr">
-        <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K235" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L235" s="2" t="inlineStr"/>
-      <c r="M235" s="3" t="inlineStr"/>
+          <t>Low / cosmetic</t>
+        </is>
+      </c>
+      <c r="J235" s="5" t="inlineStr"/>
+      <c r="K235" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L235" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M235" s="3" t="inlineStr">
+        <is>
+          <t>24fd7c273</t>
+        </is>
+      </c>
       <c r="N235" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
         </is>
       </c>
     </row>
@@ -13988,7 +13980,7 @@
       </c>
       <c r="B236" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
+          <t>CLEAN-2</t>
         </is>
       </c>
       <c r="C236" s="10" t="inlineStr">
@@ -13998,37 +13990,37 @@
       </c>
       <c r="D236" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E236" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
         </is>
       </c>
       <c r="F236" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
         </is>
       </c>
       <c r="G236" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>5 min after answer</t>
         </is>
       </c>
       <c r="I236" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Win: -671 lines.</t>
         </is>
       </c>
       <c r="J236" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
+          <t>Standard data-migration retention practice.</t>
         </is>
       </c>
       <c r="K236" s="14" t="inlineStr">
@@ -14050,109 +14042,109 @@
       </c>
       <c r="B237" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C237" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C237" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D237" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E237" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
         </is>
       </c>
       <c r="F237" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
         </is>
       </c>
       <c r="G237" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>hours-days each</t>
         </is>
       </c>
       <c r="I237" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win varies; defer until PERF-7 measured.</t>
         </is>
       </c>
       <c r="J237" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K237" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K237" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="L237" s="2" t="inlineStr"/>
       <c r="M237" s="3" t="inlineStr"/>
       <c r="N237" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="238" ht="75" customHeight="1">
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="45" customHeight="1">
       <c r="A238" s="2" t="n">
         <v>237</v>
       </c>
       <c r="B238" s="3" t="inlineStr">
         <is>
-          <t>MOD-2</t>
-        </is>
-      </c>
-      <c r="C238" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C238" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D238" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E238" s="6" t="inlineStr">
         <is>
-          <t>Pixel-diff regression baseline</t>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
         </is>
       </c>
       <c r="F238" s="5" t="inlineStr">
         <is>
-          <t>After modularization, no automated visual-regression catch.</t>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
         </is>
       </c>
       <c r="G238" s="5" t="inlineStr">
         <is>
-          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
         </is>
       </c>
       <c r="H238" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I238" s="5" t="inlineStr">
         <is>
-          <t>Win: catches accidental layout regressions.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J238" s="5" t="inlineStr">
         <is>
-          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+          <t>Agents skim and miss post-filter subset analysis.</t>
         </is>
       </c>
       <c r="K238" s="15" t="inlineStr">
@@ -14160,147 +14152,209 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L238" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
+      <c r="L238" s="2" t="inlineStr"/>
       <c r="M238" s="3" t="inlineStr"/>
       <c r="N238" s="8" t="inlineStr">
         <is>
-          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="239" ht="195" customHeight="1">
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="75" customHeight="1">
       <c r="A239" s="2" t="n">
         <v>238</v>
       </c>
       <c r="B239" s="3" t="inlineStr">
         <is>
+          <t>MOD-2</t>
+        </is>
+      </c>
+      <c r="C239" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D239" s="5" t="inlineStr">
+        <is>
+          <t>UI / Modularization</t>
+        </is>
+      </c>
+      <c r="E239" s="6" t="inlineStr">
+        <is>
+          <t>Pixel-diff regression baseline</t>
+        </is>
+      </c>
+      <c r="F239" s="5" t="inlineStr">
+        <is>
+          <t>After modularization, no automated visual-regression catch.</t>
+        </is>
+      </c>
+      <c r="G239" s="5" t="inlineStr">
+        <is>
+          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>2-3 hrs</t>
+        </is>
+      </c>
+      <c r="I239" s="5" t="inlineStr">
+        <is>
+          <t>Win: catches accidental layout regressions.</t>
+        </is>
+      </c>
+      <c r="J239" s="5" t="inlineStr">
+        <is>
+          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+        </is>
+      </c>
+      <c r="K239" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L239" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="M239" s="3" t="inlineStr"/>
+      <c r="N239" s="8" t="inlineStr">
+        <is>
+          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="195" customHeight="1">
+      <c r="A240" s="2" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
           <t>OB-CONFLUENCE-PROPOSAL-REJECTED</t>
         </is>
       </c>
-      <c r="C239" s="10" t="inlineStr">
+      <c r="C240" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D239" s="5" t="inlineStr">
+      <c r="D240" s="5" t="inlineStr">
         <is>
           <t>Signals / Cross-Check</t>
         </is>
       </c>
-      <c r="E239" s="6" t="inlineStr">
+      <c r="E240" s="6" t="inlineStr">
         <is>
           <t>OB-confluence Wilson bump + OB-aware stop — proposals KILLED by backtest evidence</t>
         </is>
       </c>
-      <c r="F239" s="5" t="inlineStr">
+      <c r="F240" s="5" t="inlineStr">
         <is>
           <t>User asked 2026-05-12 to ship #2 (Wilson-bump score factor for bullish OB confluence within 5% of entry) and #5 (OB-low as stop instead of 1.25xATR). Per Principle 1 / Principle 7, ran post-hoc validation: scripts/validate_ob_confluence.py retroactively tags every closed trade from existing portfolio_backtest outputs with SMC state at entry date, computes Wilson 95% LB per subset.
 RESULT (750-day backtest · n=384): Bull OB confluence within 5% of entry DECREASES Wilson LB by -8.6pp (14.6% vs baseline 23.1%). BOS-bullish boost: -3.4pp. SMC-bullish direction boost: -3.6pp. Per #5 simulation, 35 of 39 (90%) OB-low-as-stop would have loosened the stop; 25 of those still ended in losses (looser stops do not rescue broken setups, they extend exposure).
 Principle 4 fires: proposals FALSIFIED, killed permanently (not retuned). Doing the change without this validation would have introduced a 6-9pp Wilson-LB drag on every BUY signal.</t>
         </is>
       </c>
-      <c r="G239" s="5" t="inlineStr">
+      <c r="G240" s="5" t="inlineStr">
         <is>
           <t>Built scripts/validate_ob_confluence.py to retroactively run smart_money.score_smc() on the historical OHLCV at each trade's entry date, tag with OB-confluence + BOS + CHoCH flags, compute Wilson 95% LB per subset, and apply Principle 1 gates (n&gt;=30, lift&gt;=5pp). Cross-validated on 250d (n=142) and 750d (n=384) backtest outputs. Both agree: NO EDGE.</t>
         </is>
       </c>
-      <c r="H239" s="2" t="inlineStr">
+      <c r="H240" s="2" t="inlineStr">
         <is>
           <t>Days of work avoided (would have shipped a degrading change).</t>
         </is>
       </c>
-      <c r="I239" s="5" t="inlineStr">
+      <c r="I240" s="5" t="inlineStr">
         <is>
           <t>Mechanism (Principle 2): institutional OBs are supposed to mark re-add zones for smart money. Falsification (Principle 4): if the data doesn't show OB-confluent trades winning more, the mechanism either doesn't exist for retail-accessible OB detection at daily resolution OR is already priced into our 5-pillar score. Either way: ship nothing. The proposals are dead. Win: prevented a 6-9pp Wilson-LB drag from being added to live scoring. Lost: nothing — we didn't change live scoring, no opportunity cost.</t>
         </is>
       </c>
-      <c r="J239" s="5" t="inlineStr">
+      <c r="J240" s="5" t="inlineStr">
         <is>
           <t>Validator script is reusable infrastructure. Re-run any time the SMC detection logic or score thresholds change. NOTE: baseline WR in 750d backtest is 27.3% (low) — the absolute level reflects backtest-window-specific market conditions; the SUBSET comparisons are valid regardless because they share the same baseline. Do not interpret 23.1% Wilson LB as a system-level edge — that's a separate question. This validation answers ONLY: does OB-confluence improve selection within whatever the system already does.</t>
         </is>
       </c>
-      <c r="K239" s="15" t="inlineStr">
+      <c r="K240" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L239" s="2" t="inlineStr">
+      <c r="L240" s="2" t="inlineStr">
         <is>
           <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="M239" s="3" t="inlineStr"/>
-      <c r="N239" s="8" t="inlineStr">
-        <is>
-          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="240" ht="90" customHeight="1">
-      <c r="A240" s="2" t="n">
-        <v>239</v>
-      </c>
-      <c r="B240" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C240" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="D240" s="5" t="inlineStr">
-        <is>
-          <t>Data / Universe</t>
-        </is>
-      </c>
-      <c r="E240" s="6" t="inlineStr">
-        <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
-        </is>
-      </c>
-      <c r="F240" s="5" t="inlineStr">
-        <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
-        </is>
-      </c>
-      <c r="G240" s="5" t="inlineStr">
-        <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
-        </is>
-      </c>
-      <c r="H240" s="2" t="inlineStr">
-        <is>
-          <t>$$ + 1 day</t>
-        </is>
-      </c>
-      <c r="I240" s="5" t="inlineStr">
-        <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
-        </is>
-      </c>
-      <c r="J240" s="5" t="inlineStr">
-        <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K240" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L240" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M240" s="3" t="inlineStr"/>
       <c r="N240" s="8" t="inlineStr">
+        <is>
+          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="90" customHeight="1">
+      <c r="A241" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C241" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D241" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E241" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F241" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G241" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I241" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J241" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K241" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L241" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M241" s="3" t="inlineStr"/>
+      <c r="N241" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -14405,10 +14459,10 @@
         <v>70</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="5">
@@ -14462,10 +14516,10 @@
         <v>86</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
   </sheetData>

</xml_diff>